<commit_message>
chore(mappa): aggiornamento manuale 2026-05-19-0930
</commit_message>
<xml_diff>
--- a/Milano_2027.xlsx
+++ b/Milano_2027.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scarg\Dropbox\PNE Simone\Guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D045F1-719B-450B-87A8-03F49B5848E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685A5632-66A0-4875-9EBD-C59EE69826CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="665" xr2:uid="{0118EB4B-1337-43BA-A7E3-0EBAC20BAF10}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2115" uniqueCount="959">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2116" uniqueCount="959">
   <si>
     <t>Recensore</t>
   </si>
@@ -2364,9 +2364,6 @@
     <t>345/0229180</t>
   </si>
   <si>
-    <t>1 ceviche, 1 piatto tipico, kombucha o calice di vino</t>
-  </si>
-  <si>
     <t>Via Raffaello Sanzio, 22</t>
   </si>
   <si>
@@ -2914,6 +2911,9 @@
   </si>
   <si>
     <t>1 fritto, 1 pizza stile romano, 1 pizza stile contemporaneo, farciture diverse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">due piatti (no stuzzichini o piatti semplici)+ calice di vino </t>
   </si>
 </sst>
 </file>
@@ -3730,15 +3730,15 @@
       </c>
       <c r="F4" s="9">
         <f>+AD6</f>
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="G4" s="9">
         <f>+AF6</f>
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="H4" s="7">
         <f>+E4-G4</f>
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="I4" s="24" t="s">
         <v>16</v>
@@ -3760,15 +3760,15 @@
       </c>
       <c r="F5" s="11">
         <f>+F3+F4</f>
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G5" s="11">
         <f>+G3+G4</f>
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="H5" s="11">
         <f>+H3+H4</f>
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="I5" s="25" t="s">
         <v>43</v>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="AD6" s="2">
         <f t="shared" si="1"/>
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="AE6" s="2">
         <f t="shared" si="1"/>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="AF6" s="2">
         <f t="shared" si="1"/>
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="AG6" s="2">
         <f t="shared" si="1"/>
@@ -3912,7 +3912,7 @@
         <v>42</v>
       </c>
       <c r="K7" s="37" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="L7" s="37" t="s">
         <v>19</v>
@@ -4027,10 +4027,10 @@
         <v>205</v>
       </c>
       <c r="M8" s="35" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="N8" s="35" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="O8" s="36"/>
       <c r="P8" s="36"/>
@@ -4140,7 +4140,7 @@
         <v>40</v>
       </c>
       <c r="N9" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O9" s="33">
         <v>1</v>
@@ -4364,7 +4364,7 @@
         <v>206</v>
       </c>
       <c r="N11" s="35" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="O11" s="36"/>
       <c r="P11" s="36"/>
@@ -4471,10 +4471,10 @@
         <v>160</v>
       </c>
       <c r="M12" s="35" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="N12" s="35" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="O12" s="36"/>
       <c r="P12" s="36"/>
@@ -4554,7 +4554,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="35" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="E13" s="35" t="s">
         <v>260</v>
@@ -4581,10 +4581,10 @@
         <v>210</v>
       </c>
       <c r="M13" s="35" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="N13" s="35" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="O13" s="36"/>
       <c r="P13" s="36"/>
@@ -4694,7 +4694,7 @@
         <v>40</v>
       </c>
       <c r="N14" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O14" s="33">
         <v>1</v>
@@ -4802,13 +4802,13 @@
         <v>325</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="M15" s="35" t="s">
         <v>741</v>
       </c>
       <c r="N15" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O15" s="36"/>
       <c r="P15" s="36"/>
@@ -4912,7 +4912,7 @@
         <v>328</v>
       </c>
       <c r="L16" s="20" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="M16" s="21" t="s">
         <v>742</v>
@@ -5023,10 +5023,10 @@
         <v>170</v>
       </c>
       <c r="M17" s="35" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="N17" s="35" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="O17" s="36"/>
       <c r="P17" s="36"/>
@@ -5136,7 +5136,7 @@
         <v>40</v>
       </c>
       <c r="N18" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O18" s="33">
         <v>1</v>
@@ -5235,7 +5235,7 @@
         <v>165</v>
       </c>
       <c r="I19" s="34" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="J19" s="34">
         <v>99</v>
@@ -5244,13 +5244,13 @@
         <v>328</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="M19" s="35" t="s">
         <v>744</v>
       </c>
       <c r="N19" s="35" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="O19" s="36"/>
       <c r="P19" s="36"/>
@@ -5354,7 +5354,7 @@
         <v>328</v>
       </c>
       <c r="L20" s="20" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M20" s="21" t="s">
         <v>206</v>
@@ -5465,10 +5465,10 @@
         <v>75</v>
       </c>
       <c r="M21" s="35" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="N21" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O21" s="36"/>
       <c r="P21" s="36"/>
@@ -5554,10 +5554,10 @@
         <v>468</v>
       </c>
       <c r="F22" s="35" t="s">
+        <v>840</v>
+      </c>
+      <c r="G22" s="35" t="s">
         <v>841</v>
-      </c>
-      <c r="G22" s="35" t="s">
-        <v>842</v>
       </c>
       <c r="H22" s="35" t="s">
         <v>165</v>
@@ -5578,7 +5578,7 @@
         <v>206</v>
       </c>
       <c r="N22" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O22" s="36"/>
       <c r="P22" s="36"/>
@@ -5688,7 +5688,7 @@
         <v>206</v>
       </c>
       <c r="N23" s="35" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="O23" s="36"/>
       <c r="P23" s="36"/>
@@ -5783,7 +5783,7 @@
         <v>165</v>
       </c>
       <c r="I24" s="34" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="J24" s="34">
         <v>99</v>
@@ -5795,10 +5795,10 @@
         <v>45</v>
       </c>
       <c r="M24" s="35" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="N24" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O24" s="36"/>
       <c r="P24" s="36"/>
@@ -5902,13 +5902,13 @@
         <v>330</v>
       </c>
       <c r="L25" s="34" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="M25" s="35" t="s">
         <v>743</v>
       </c>
       <c r="N25" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O25" s="36"/>
       <c r="P25" s="36"/>
@@ -6012,10 +6012,10 @@
         <v>329</v>
       </c>
       <c r="L26" s="20" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="M26" s="21" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="N26" s="21"/>
       <c r="O26" s="7"/>
@@ -6126,7 +6126,7 @@
         <v>206</v>
       </c>
       <c r="N27" s="32" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="O27" s="33">
         <v>1</v>
@@ -6348,7 +6348,7 @@
         <v>206</v>
       </c>
       <c r="N29" s="35" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="O29" s="36"/>
       <c r="P29" s="36"/>
@@ -6455,10 +6455,10 @@
         <v>150</v>
       </c>
       <c r="M30" s="35" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="N30" s="35" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="O30" s="36"/>
       <c r="P30" s="36"/>
@@ -6565,10 +6565,10 @@
         <v>90</v>
       </c>
       <c r="M31" s="35" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="N31" s="35" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="O31" s="36"/>
       <c r="P31" s="36"/>
@@ -6678,7 +6678,7 @@
         <v>344</v>
       </c>
       <c r="N32" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O32" s="36"/>
       <c r="P32" s="36"/>
@@ -6758,7 +6758,7 @@
         <v>2</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="E33" s="21" t="s">
         <v>262</v>
@@ -6773,7 +6773,7 @@
         <v>165</v>
       </c>
       <c r="I33" s="20" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="J33" s="20">
         <v>4</v>
@@ -6785,7 +6785,7 @@
         <v>130</v>
       </c>
       <c r="M33" s="21" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="N33" s="21"/>
       <c r="O33" s="7"/>
@@ -6896,7 +6896,7 @@
         <v>40</v>
       </c>
       <c r="N34" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O34" s="33">
         <v>1</v>
@@ -7007,10 +7007,10 @@
         <v>45</v>
       </c>
       <c r="M35" s="32" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="N35" s="32" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="O35" s="33">
         <v>1</v>
@@ -7230,7 +7230,7 @@
         <v>601</v>
       </c>
       <c r="N37" s="35" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="O37" s="36"/>
       <c r="P37" s="36"/>
@@ -7340,7 +7340,7 @@
         <v>602</v>
       </c>
       <c r="N38" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O38" s="33">
         <v>1</v>
@@ -7424,7 +7424,7 @@
         <v>3</v>
       </c>
       <c r="D39" s="21" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="E39" s="21" t="s">
         <v>501</v>
@@ -7448,7 +7448,7 @@
         <v>329</v>
       </c>
       <c r="L39" s="20" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="M39" s="21" t="s">
         <v>602</v>
@@ -7522,50 +7522,52 @@
       </c>
     </row>
     <row r="40" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="34">
-        <v>0</v>
-      </c>
-      <c r="B40" s="34">
-        <v>1</v>
-      </c>
-      <c r="C40" s="34">
+      <c r="A40" s="31">
+        <v>0</v>
+      </c>
+      <c r="B40" s="31">
+        <v>1</v>
+      </c>
+      <c r="C40" s="31">
         <v>3</v>
       </c>
-      <c r="D40" s="35" t="s">
+      <c r="D40" s="32" t="s">
         <v>514</v>
       </c>
-      <c r="E40" s="35" t="s">
+      <c r="E40" s="32" t="s">
         <v>679</v>
       </c>
-      <c r="F40" s="35" t="s">
+      <c r="F40" s="32" t="s">
         <v>515</v>
       </c>
-      <c r="G40" s="35" t="s">
+      <c r="G40" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="H40" s="35" t="s">
+      <c r="H40" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I40" s="34" t="s">
+      <c r="I40" s="31" t="s">
         <v>516</v>
       </c>
-      <c r="J40" s="34">
+      <c r="J40" s="31">
         <v>8</v>
       </c>
-      <c r="K40" s="34" t="s">
+      <c r="K40" s="31" t="s">
         <v>326</v>
       </c>
-      <c r="L40" s="34" t="s">
-        <v>864</v>
-      </c>
-      <c r="M40" s="35" t="s">
+      <c r="L40" s="31" t="s">
+        <v>863</v>
+      </c>
+      <c r="M40" s="32" t="s">
         <v>746</v>
       </c>
-      <c r="N40" s="35" t="s">
-        <v>917</v>
-      </c>
-      <c r="O40" s="36"/>
-      <c r="P40" s="36"/>
+      <c r="N40" s="32" t="s">
+        <v>919</v>
+      </c>
+      <c r="O40" s="33">
+        <v>1</v>
+      </c>
+      <c r="P40" s="33"/>
       <c r="R40" s="2">
         <f t="shared" si="23"/>
         <v>0</v>
@@ -7612,7 +7614,7 @@
       </c>
       <c r="AD40" s="2">
         <f t="shared" si="34"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE40" s="2">
         <f t="shared" si="19"/>
@@ -7620,7 +7622,7 @@
       </c>
       <c r="AF40" s="2">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG40" s="2">
         <f t="shared" si="21"/>
@@ -7666,13 +7668,13 @@
         <v>326</v>
       </c>
       <c r="L41" s="34" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="M41" s="35" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="N41" s="35" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="O41" s="36"/>
       <c r="P41" s="36"/>
@@ -7782,7 +7784,7 @@
         <v>763</v>
       </c>
       <c r="N42" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O42" s="36"/>
       <c r="P42" s="36"/>
@@ -7892,7 +7894,7 @@
         <v>746</v>
       </c>
       <c r="N43" s="32" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="O43" s="33">
         <v>1</v>
@@ -8004,7 +8006,7 @@
         <v>602</v>
       </c>
       <c r="N44" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O44" s="36"/>
       <c r="P44" s="36"/>
@@ -8114,7 +8116,7 @@
         <v>512</v>
       </c>
       <c r="N45" s="32" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="O45" s="33">
         <v>1</v>
@@ -8196,13 +8198,13 @@
         <v>3</v>
       </c>
       <c r="D46" s="35" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="E46" s="35" t="s">
         <v>259</v>
       </c>
       <c r="F46" s="35" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="G46" s="35" t="s">
         <v>103</v>
@@ -8211,7 +8213,7 @@
         <v>165</v>
       </c>
       <c r="I46" s="34" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="J46" s="34">
         <v>6</v>
@@ -8223,10 +8225,10 @@
         <v>70</v>
       </c>
       <c r="M46" s="35" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="N46" s="35" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="O46" s="36"/>
       <c r="P46" s="36"/>
@@ -8315,7 +8317,7 @@
         <v>613</v>
       </c>
       <c r="G47" s="35" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="H47" s="35" t="s">
         <v>165</v>
@@ -8336,7 +8338,7 @@
         <v>746</v>
       </c>
       <c r="N47" s="35" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="O47" s="36"/>
       <c r="P47" s="36"/>
@@ -8446,7 +8448,7 @@
         <v>206</v>
       </c>
       <c r="N48" s="35" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="O48" s="36"/>
       <c r="P48" s="36"/>
@@ -8556,7 +8558,7 @@
         <v>266</v>
       </c>
       <c r="N49" s="32" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="O49" s="33">
         <v>1</v>
@@ -8776,7 +8778,7 @@
         <v>644</v>
       </c>
       <c r="N51" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O51" s="36"/>
       <c r="P51" s="36"/>
@@ -8862,7 +8864,7 @@
         <v>259</v>
       </c>
       <c r="F52" s="35" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="G52" s="35" t="s">
         <v>736</v>
@@ -8886,7 +8888,7 @@
         <v>734</v>
       </c>
       <c r="N52" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O52" s="36"/>
       <c r="P52" s="36"/>
@@ -8996,7 +8998,7 @@
         <v>741</v>
       </c>
       <c r="N53" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O53" s="36"/>
       <c r="P53" s="36"/>
@@ -9103,7 +9105,7 @@
         <v>50</v>
       </c>
       <c r="M54" s="21" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="N54" s="21"/>
       <c r="O54" s="7"/>
@@ -9211,10 +9213,10 @@
         <v>345</v>
       </c>
       <c r="M55" s="32" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="N55" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O55" s="33">
         <v>1</v>
@@ -9328,7 +9330,7 @@
         <v>266</v>
       </c>
       <c r="N56" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O56" s="36"/>
       <c r="P56" s="36"/>
@@ -9516,13 +9518,13 @@
         <v>5</v>
       </c>
       <c r="D58" s="35" t="s">
+        <v>894</v>
+      </c>
+      <c r="E58" s="35" t="s">
+        <v>897</v>
+      </c>
+      <c r="F58" s="35" t="s">
         <v>895</v>
-      </c>
-      <c r="E58" s="35" t="s">
-        <v>898</v>
-      </c>
-      <c r="F58" s="35" t="s">
-        <v>896</v>
       </c>
       <c r="G58" s="35" t="s">
         <v>403</v>
@@ -9531,7 +9533,7 @@
         <v>165</v>
       </c>
       <c r="I58" s="34" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="J58" s="34"/>
       <c r="K58" s="34" t="s">
@@ -9541,10 +9543,10 @@
         <v>55</v>
       </c>
       <c r="M58" s="35" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="N58" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O58" s="36"/>
       <c r="P58" s="36"/>
@@ -9624,13 +9626,13 @@
         <v>5</v>
       </c>
       <c r="D59" s="32" t="s">
+        <v>879</v>
+      </c>
+      <c r="E59" s="32" t="s">
+        <v>808</v>
+      </c>
+      <c r="F59" s="32" t="s">
         <v>880</v>
-      </c>
-      <c r="E59" s="32" t="s">
-        <v>809</v>
-      </c>
-      <c r="F59" s="32" t="s">
-        <v>881</v>
       </c>
       <c r="G59" s="32" t="s">
         <v>309</v>
@@ -9639,7 +9641,7 @@
         <v>165</v>
       </c>
       <c r="I59" s="31" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="J59" s="31"/>
       <c r="K59" s="31" t="s">
@@ -9649,10 +9651,10 @@
         <v>50</v>
       </c>
       <c r="M59" s="32" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="N59" s="32" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="O59" s="33">
         <v>1</v>
@@ -9734,13 +9736,13 @@
         <v>5</v>
       </c>
       <c r="D60" s="21" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="E60" s="21" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F60" s="21" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="G60" s="21" t="s">
         <v>93</v>
@@ -9749,7 +9751,7 @@
         <v>165</v>
       </c>
       <c r="I60" s="20" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="J60" s="20">
         <v>8</v>
@@ -9761,7 +9763,7 @@
         <v>50</v>
       </c>
       <c r="M60" s="21" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="N60" s="21"/>
       <c r="O60" s="7"/>
@@ -9842,13 +9844,13 @@
         <v>5</v>
       </c>
       <c r="D61" s="32" t="s">
+        <v>876</v>
+      </c>
+      <c r="E61" s="32" t="s">
+        <v>808</v>
+      </c>
+      <c r="F61" s="32" t="s">
         <v>877</v>
-      </c>
-      <c r="E61" s="32" t="s">
-        <v>809</v>
-      </c>
-      <c r="F61" s="32" t="s">
-        <v>878</v>
       </c>
       <c r="G61" s="32" t="s">
         <v>370</v>
@@ -9857,7 +9859,7 @@
         <v>165</v>
       </c>
       <c r="I61" s="31" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="J61" s="31"/>
       <c r="K61" s="31" t="s">
@@ -9870,7 +9872,7 @@
         <v>420</v>
       </c>
       <c r="N61" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O61" s="33">
         <v>1</v>
@@ -9984,7 +9986,7 @@
         <v>266</v>
       </c>
       <c r="N62" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O62" s="33">
         <v>1</v>
@@ -10096,7 +10098,7 @@
         <v>420</v>
       </c>
       <c r="N63" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O63" s="33">
         <v>1</v>
@@ -10208,7 +10210,7 @@
         <v>420</v>
       </c>
       <c r="N64" s="35" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="O64" s="36"/>
       <c r="P64" s="36"/>
@@ -10315,10 +10317,10 @@
         <v>341</v>
       </c>
       <c r="M65" s="32" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="N65" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O65" s="33">
         <v>1</v>
@@ -10430,7 +10432,7 @@
         <v>498</v>
       </c>
       <c r="N66" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O66" s="36"/>
       <c r="P66" s="36"/>
@@ -10648,7 +10650,7 @@
         <v>420</v>
       </c>
       <c r="N68" s="35" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="O68" s="36"/>
       <c r="P68" s="36"/>
@@ -10728,7 +10730,7 @@
         <v>5</v>
       </c>
       <c r="D69" s="35" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="E69" s="35" t="s">
         <v>264</v>
@@ -10758,7 +10760,7 @@
         <v>266</v>
       </c>
       <c r="N69" s="35" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="O69" s="36"/>
       <c r="P69" s="36"/>
@@ -10838,13 +10840,13 @@
         <v>5</v>
       </c>
       <c r="D70" s="21" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="E70" s="21" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F70" s="21" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="G70" s="21" t="s">
         <v>117</v>
@@ -10853,7 +10855,7 @@
         <v>165</v>
       </c>
       <c r="I70" s="20" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="J70" s="20">
         <v>1</v>
@@ -10946,13 +10948,13 @@
         <v>5</v>
       </c>
       <c r="D71" s="21" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="E71" s="21" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F71" s="21" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="G71" s="21" t="s">
         <v>96</v>
@@ -10961,7 +10963,7 @@
         <v>165</v>
       </c>
       <c r="I71" s="20" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="J71" s="20">
         <v>3</v>
@@ -11054,13 +11056,13 @@
         <v>6</v>
       </c>
       <c r="D72" s="32" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="E72" s="32" t="s">
         <v>261</v>
       </c>
       <c r="F72" s="32" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="G72" s="32" t="s">
         <v>521</v>
@@ -11069,7 +11071,7 @@
         <v>165</v>
       </c>
       <c r="I72" s="31" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="J72" s="31">
         <v>99</v>
@@ -11084,7 +11086,7 @@
         <v>40</v>
       </c>
       <c r="N72" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O72" s="33">
         <v>1</v>
@@ -11268,48 +11270,50 @@
       </c>
     </row>
     <row r="74" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="34">
-        <v>0</v>
-      </c>
-      <c r="B74" s="34">
-        <v>1</v>
-      </c>
-      <c r="C74" s="34">
+      <c r="A74" s="31">
+        <v>0</v>
+      </c>
+      <c r="B74" s="31">
+        <v>1</v>
+      </c>
+      <c r="C74" s="31">
         <v>6</v>
       </c>
-      <c r="D74" s="35" t="s">
+      <c r="D74" s="32" t="s">
         <v>227</v>
       </c>
-      <c r="E74" s="35" t="s">
+      <c r="E74" s="32" t="s">
         <v>677</v>
       </c>
-      <c r="F74" s="35" t="s">
+      <c r="F74" s="32" t="s">
         <v>669</v>
       </c>
-      <c r="G74" s="35" t="s">
+      <c r="G74" s="32" t="s">
         <v>670</v>
       </c>
-      <c r="H74" s="35" t="s">
+      <c r="H74" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I74" s="34" t="s">
+      <c r="I74" s="31" t="s">
         <v>671</v>
       </c>
-      <c r="J74" s="34"/>
-      <c r="K74" s="34" t="s">
+      <c r="J74" s="31"/>
+      <c r="K74" s="31" t="s">
         <v>332</v>
       </c>
-      <c r="L74" s="34">
+      <c r="L74" s="31">
         <v>45</v>
       </c>
-      <c r="M74" s="35" t="s">
+      <c r="M74" s="32" t="s">
         <v>757</v>
       </c>
-      <c r="N74" s="35" t="s">
-        <v>902</v>
-      </c>
-      <c r="O74" s="36"/>
-      <c r="P74" s="36"/>
+      <c r="N74" s="32" t="s">
+        <v>906</v>
+      </c>
+      <c r="O74" s="33">
+        <v>1</v>
+      </c>
+      <c r="P74" s="33"/>
       <c r="R74" s="2">
         <f t="shared" si="23"/>
         <v>0</v>
@@ -11356,7 +11360,7 @@
       </c>
       <c r="AD74" s="2">
         <f t="shared" si="34"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE74" s="2">
         <f t="shared" si="19"/>
@@ -11364,7 +11368,7 @@
       </c>
       <c r="AF74" s="2">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG74" s="2">
         <f t="shared" si="21"/>
@@ -11376,50 +11380,52 @@
       </c>
     </row>
     <row r="75" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="34">
-        <v>1</v>
-      </c>
-      <c r="B75" s="34">
-        <v>1</v>
-      </c>
-      <c r="C75" s="34">
+      <c r="A75" s="31">
+        <v>1</v>
+      </c>
+      <c r="B75" s="31">
+        <v>1</v>
+      </c>
+      <c r="C75" s="31">
         <v>6</v>
       </c>
-      <c r="D75" s="35" t="s">
+      <c r="D75" s="32" t="s">
         <v>227</v>
       </c>
-      <c r="E75" s="35" t="s">
+      <c r="E75" s="32" t="s">
         <v>677</v>
       </c>
-      <c r="F75" s="35" t="s">
+      <c r="F75" s="32" t="s">
         <v>228</v>
       </c>
-      <c r="G75" s="35" t="s">
+      <c r="G75" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="H75" s="35" t="s">
+      <c r="H75" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I75" s="34" t="s">
+      <c r="I75" s="31" t="s">
         <v>229</v>
       </c>
-      <c r="J75" s="34">
+      <c r="J75" s="31">
         <v>6</v>
       </c>
-      <c r="K75" s="34" t="s">
+      <c r="K75" s="31" t="s">
         <v>332</v>
       </c>
-      <c r="L75" s="34">
+      <c r="L75" s="31">
         <v>45</v>
       </c>
-      <c r="M75" s="35" t="s">
+      <c r="M75" s="32" t="s">
         <v>757</v>
       </c>
-      <c r="N75" s="35" t="s">
-        <v>902</v>
-      </c>
-      <c r="O75" s="36"/>
-      <c r="P75" s="36"/>
+      <c r="N75" s="32" t="s">
+        <v>906</v>
+      </c>
+      <c r="O75" s="33">
+        <v>1</v>
+      </c>
+      <c r="P75" s="33"/>
       <c r="R75" s="2">
         <f t="shared" si="23"/>
         <v>0</v>
@@ -11466,7 +11472,7 @@
       </c>
       <c r="AD75" s="2">
         <f t="shared" si="34"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE75" s="2">
         <f t="shared" si="19"/>
@@ -11521,10 +11527,10 @@
         <v>35</v>
       </c>
       <c r="M76" s="32" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="N76" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O76" s="33">
         <v>1</v>
@@ -11633,10 +11639,10 @@
         <v>40</v>
       </c>
       <c r="M77" s="32" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="N77" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O77" s="33">
         <v>1</v>
@@ -11748,7 +11754,7 @@
         <v>40</v>
       </c>
       <c r="N78" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O78" s="33">
         <v>1</v>
@@ -11862,7 +11868,7 @@
         <v>206</v>
       </c>
       <c r="N79" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O79" s="36"/>
       <c r="P79" s="36"/>
@@ -12067,7 +12073,7 @@
         <v>165</v>
       </c>
       <c r="I81" s="31" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="J81" s="31">
         <v>3</v>
@@ -12082,7 +12088,7 @@
         <v>770</v>
       </c>
       <c r="N81" s="32" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="O81" s="33">
         <v>1</v>
@@ -12188,13 +12194,13 @@
         <v>329</v>
       </c>
       <c r="L82" s="34" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="M82" s="35" t="s">
         <v>703</v>
       </c>
       <c r="N82" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O82" s="36"/>
       <c r="P82" s="36"/>
@@ -12304,7 +12310,7 @@
         <v>754</v>
       </c>
       <c r="N83" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O83" s="33">
         <v>1</v>
@@ -12714,7 +12720,7 @@
         <v>577</v>
       </c>
       <c r="F87" s="35" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="G87" s="35" t="s">
         <v>544</v>
@@ -12738,7 +12744,7 @@
         <v>748</v>
       </c>
       <c r="N87" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O87" s="36"/>
       <c r="P87" s="36"/>
@@ -12808,50 +12814,52 @@
       </c>
     </row>
     <row r="88" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="34">
-        <v>0</v>
-      </c>
-      <c r="B88" s="34">
-        <v>1</v>
-      </c>
-      <c r="C88" s="34">
+      <c r="A88" s="31">
+        <v>0</v>
+      </c>
+      <c r="B88" s="31">
+        <v>1</v>
+      </c>
+      <c r="C88" s="31">
         <v>6</v>
       </c>
-      <c r="D88" s="35" t="s">
+      <c r="D88" s="32" t="s">
         <v>360</v>
       </c>
-      <c r="E88" s="35" t="s">
+      <c r="E88" s="32" t="s">
         <v>578</v>
       </c>
-      <c r="F88" s="35" t="s">
+      <c r="F88" s="32" t="s">
         <v>136</v>
       </c>
-      <c r="G88" s="35" t="s">
+      <c r="G88" s="32" t="s">
         <v>137</v>
       </c>
-      <c r="H88" s="35" t="s">
+      <c r="H88" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I88" s="34" t="s">
+      <c r="I88" s="31" t="s">
         <v>184</v>
       </c>
-      <c r="J88" s="34">
-        <v>1</v>
-      </c>
-      <c r="K88" s="34" t="s">
+      <c r="J88" s="31">
+        <v>1</v>
+      </c>
+      <c r="K88" s="31" t="s">
         <v>378</v>
       </c>
-      <c r="L88" s="34">
+      <c r="L88" s="31">
         <v>92</v>
       </c>
-      <c r="M88" s="35" t="s">
-        <v>788</v>
-      </c>
-      <c r="N88" s="35" t="s">
-        <v>905</v>
-      </c>
-      <c r="O88" s="36"/>
-      <c r="P88" s="36"/>
+      <c r="M88" s="32" t="s">
+        <v>787</v>
+      </c>
+      <c r="N88" s="32" t="s">
+        <v>914</v>
+      </c>
+      <c r="O88" s="33">
+        <v>1</v>
+      </c>
+      <c r="P88" s="33"/>
       <c r="R88" s="2">
         <f t="shared" si="39"/>
         <v>1</v>
@@ -12898,7 +12906,7 @@
       </c>
       <c r="AD88" s="2">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE88" s="2">
         <f t="shared" si="35"/>
@@ -12906,7 +12914,7 @@
       </c>
       <c r="AF88" s="2">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG88" s="2">
         <f t="shared" si="37"/>
@@ -13066,7 +13074,7 @@
         <v>298</v>
       </c>
       <c r="N90" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O90" s="33">
         <v>1</v>
@@ -13178,7 +13186,7 @@
         <v>298</v>
       </c>
       <c r="N91" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O91" s="33">
         <v>1</v>
@@ -13290,7 +13298,7 @@
         <v>298</v>
       </c>
       <c r="N92" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O92" s="33">
         <v>1</v>
@@ -13402,7 +13410,7 @@
         <v>298</v>
       </c>
       <c r="N93" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O93" s="33">
         <v>1</v>
@@ -13514,7 +13522,7 @@
         <v>298</v>
       </c>
       <c r="N94" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O94" s="33">
         <v>1</v>
@@ -13626,7 +13634,7 @@
         <v>298</v>
       </c>
       <c r="N95" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O95" s="33">
         <v>1</v>
@@ -13848,7 +13856,7 @@
         <v>340</v>
       </c>
       <c r="N97" s="32" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="O97" s="33">
         <v>1</v>
@@ -13945,7 +13953,7 @@
         <v>165</v>
       </c>
       <c r="I98" s="31" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="J98" s="31">
         <v>1</v>
@@ -13960,7 +13968,7 @@
         <v>755</v>
       </c>
       <c r="N98" s="32" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="O98" s="33">
         <v>1</v>
@@ -14072,7 +14080,7 @@
         <v>755</v>
       </c>
       <c r="N99" s="32" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="O99" s="33">
         <v>1</v>
@@ -14184,7 +14192,7 @@
         <v>755</v>
       </c>
       <c r="N100" s="32" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="O100" s="33">
         <v>1</v>
@@ -14296,7 +14304,7 @@
         <v>40</v>
       </c>
       <c r="N101" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O101" s="33">
         <v>1</v>
@@ -14410,7 +14418,7 @@
         <v>40</v>
       </c>
       <c r="N102" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O102" s="33">
         <v>1</v>
@@ -14500,7 +14508,7 @@
         <v>32</v>
       </c>
       <c r="F103" s="32" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="G103" s="32" t="s">
         <v>124</v>
@@ -14509,7 +14517,7 @@
         <v>165</v>
       </c>
       <c r="I103" s="31" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="J103" s="31">
         <v>99</v>
@@ -14524,7 +14532,7 @@
         <v>40</v>
       </c>
       <c r="N103" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O103" s="33">
         <v>1</v>
@@ -14614,7 +14622,7 @@
         <v>32</v>
       </c>
       <c r="F104" s="32" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="G104" s="32" t="s">
         <v>103</v>
@@ -14623,7 +14631,7 @@
         <v>165</v>
       </c>
       <c r="I104" s="31" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="J104" s="31">
         <v>2</v>
@@ -14638,7 +14646,7 @@
         <v>40</v>
       </c>
       <c r="N104" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O104" s="33">
         <v>1</v>
@@ -14752,7 +14760,7 @@
         <v>268</v>
       </c>
       <c r="N105" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O105" s="36"/>
       <c r="P105" s="36"/>
@@ -14862,7 +14870,7 @@
         <v>268</v>
       </c>
       <c r="N106" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O106" s="36"/>
       <c r="P106" s="36"/>
@@ -14942,20 +14950,20 @@
         <v>7</v>
       </c>
       <c r="D107" s="21" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="E107" s="21" t="s">
         <v>32</v>
       </c>
       <c r="F107" s="21" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="G107" s="21"/>
       <c r="H107" s="21" t="s">
         <v>165</v>
       </c>
       <c r="I107" s="20" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="J107" s="20"/>
       <c r="K107" s="20" t="s">
@@ -14965,7 +14973,7 @@
         <v>30</v>
       </c>
       <c r="M107" s="21" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="N107" s="21"/>
       <c r="O107" s="7"/>
@@ -15076,7 +15084,7 @@
         <v>651</v>
       </c>
       <c r="N108" s="35" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="O108" s="36"/>
       <c r="P108" s="36"/>
@@ -15186,7 +15194,7 @@
         <v>298</v>
       </c>
       <c r="N109" s="32" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="O109" s="33">
         <v>1</v>
@@ -15296,7 +15304,7 @@
         <v>298</v>
       </c>
       <c r="N110" s="32" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="O110" s="33">
         <v>1</v>
@@ -15408,7 +15416,7 @@
         <v>269</v>
       </c>
       <c r="N111" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O111" s="33">
         <v>1</v>
@@ -15522,7 +15530,7 @@
         <v>269</v>
       </c>
       <c r="N112" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O112" s="33">
         <v>1</v>
@@ -15606,13 +15614,13 @@
         <v>1</v>
       </c>
       <c r="D113" s="21" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="E113" s="21" t="s">
         <v>471</v>
       </c>
       <c r="F113" s="21" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="G113" s="21" t="s">
         <v>114</v>
@@ -15621,7 +15629,7 @@
         <v>165</v>
       </c>
       <c r="I113" s="20" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="J113" s="20">
         <v>99</v>
@@ -15633,7 +15641,7 @@
         <v>6</v>
       </c>
       <c r="M113" s="21" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="N113" s="21"/>
       <c r="O113" s="7"/>
@@ -15714,13 +15722,13 @@
         <v>1</v>
       </c>
       <c r="D114" s="32" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E114" s="32" t="s">
         <v>471</v>
       </c>
       <c r="F114" s="32" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="G114" s="32" t="s">
         <v>103</v>
@@ -15729,7 +15737,7 @@
         <v>165</v>
       </c>
       <c r="I114" s="31" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="J114" s="31">
         <v>2</v>
@@ -15741,10 +15749,10 @@
         <v>15</v>
       </c>
       <c r="M114" s="32" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="N114" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O114" s="33">
         <v>1</v>
@@ -15855,10 +15863,10 @@
         <v>13</v>
       </c>
       <c r="M115" s="32" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="N115" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O115" s="33">
         <v>1</v>
@@ -15969,10 +15977,10 @@
         <v>13</v>
       </c>
       <c r="M116" s="32" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="N116" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O116" s="33">
         <v>1</v>
@@ -16083,10 +16091,10 @@
         <v>13</v>
       </c>
       <c r="M117" s="32" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="N117" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O117" s="33">
         <v>1</v>
@@ -16176,10 +16184,10 @@
         <v>471</v>
       </c>
       <c r="F118" s="32" t="s">
+        <v>781</v>
+      </c>
+      <c r="G118" s="32" t="s">
         <v>782</v>
-      </c>
-      <c r="G118" s="32" t="s">
-        <v>783</v>
       </c>
       <c r="H118" s="32" t="s">
         <v>165</v>
@@ -16197,10 +16205,10 @@
         <v>13</v>
       </c>
       <c r="M118" s="32" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="N118" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O118" s="33">
         <v>1</v>
@@ -16290,10 +16298,10 @@
         <v>471</v>
       </c>
       <c r="F119" s="32" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="G119" s="32" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="H119" s="32" t="s">
         <v>165</v>
@@ -16311,10 +16319,10 @@
         <v>13</v>
       </c>
       <c r="M119" s="32" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="N119" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O119" s="33">
         <v>1</v>
@@ -16388,50 +16396,52 @@
       </c>
     </row>
     <row r="120" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="34">
-        <v>0</v>
-      </c>
-      <c r="B120" s="34">
+      <c r="A120" s="31">
+        <v>0</v>
+      </c>
+      <c r="B120" s="31">
         <v>2</v>
       </c>
-      <c r="C120" s="34">
-        <v>1</v>
-      </c>
-      <c r="D120" s="35" t="s">
+      <c r="C120" s="31">
+        <v>1</v>
+      </c>
+      <c r="D120" s="32" t="s">
         <v>666</v>
       </c>
-      <c r="E120" s="35" t="s">
+      <c r="E120" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="F120" s="35" t="s">
+      <c r="F120" s="32" t="s">
         <v>638</v>
       </c>
-      <c r="G120" s="35" t="s">
+      <c r="G120" s="32" t="s">
         <v>691</v>
       </c>
-      <c r="H120" s="35" t="s">
+      <c r="H120" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I120" s="34" t="s">
+      <c r="I120" s="31" t="s">
         <v>639</v>
       </c>
-      <c r="J120" s="34">
+      <c r="J120" s="31">
         <v>99</v>
       </c>
-      <c r="K120" s="34" t="s">
+      <c r="K120" s="31" t="s">
         <v>318</v>
       </c>
-      <c r="L120" s="34" t="s">
+      <c r="L120" s="31" t="s">
         <v>318</v>
       </c>
-      <c r="M120" s="35" t="s">
+      <c r="M120" s="32" t="s">
         <v>269</v>
       </c>
-      <c r="N120" s="35" t="s">
-        <v>902</v>
-      </c>
-      <c r="O120" s="36"/>
-      <c r="P120" s="36"/>
+      <c r="N120" s="32" t="s">
+        <v>906</v>
+      </c>
+      <c r="O120" s="33">
+        <v>1</v>
+      </c>
+      <c r="P120" s="33"/>
       <c r="R120" s="2">
         <f t="shared" si="39"/>
         <v>0</v>
@@ -16478,7 +16488,7 @@
       </c>
       <c r="AD120" s="2">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE120" s="2">
         <f t="shared" si="35"/>
@@ -16486,7 +16496,7 @@
       </c>
       <c r="AF120" s="2">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG120" s="2">
         <f t="shared" si="37"/>
@@ -16508,13 +16518,13 @@
         <v>1</v>
       </c>
       <c r="D121" s="32" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="E121" s="32" t="s">
         <v>471</v>
       </c>
       <c r="F121" s="32" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="G121" s="32" t="s">
         <v>38</v>
@@ -16523,7 +16533,7 @@
         <v>165</v>
       </c>
       <c r="I121" s="31" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="J121" s="31">
         <v>1</v>
@@ -16534,7 +16544,7 @@
       <c r="L121" s="31"/>
       <c r="M121" s="32"/>
       <c r="N121" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O121" s="33">
         <v>1</v>
@@ -16627,7 +16637,7 @@
         <v>765</v>
       </c>
       <c r="G122" s="32" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="H122" s="32" t="s">
         <v>165</v>
@@ -16646,7 +16656,7 @@
         <v>711</v>
       </c>
       <c r="N122" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O122" s="33">
         <v>1</v>
@@ -16760,7 +16770,7 @@
         <v>269</v>
       </c>
       <c r="N123" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O123" s="33">
         <v>1</v>
@@ -16874,7 +16884,7 @@
         <v>269</v>
       </c>
       <c r="N124" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O124" s="33">
         <v>1</v>
@@ -16988,7 +16998,7 @@
         <v>269</v>
       </c>
       <c r="N125" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O125" s="33">
         <v>1</v>
@@ -17102,7 +17112,7 @@
         <v>269</v>
       </c>
       <c r="N126" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O126" s="36"/>
       <c r="P126" s="36"/>
@@ -17290,13 +17300,13 @@
         <v>1</v>
       </c>
       <c r="D128" s="32" t="s">
+        <v>947</v>
+      </c>
+      <c r="E128" s="32" t="s">
         <v>948</v>
       </c>
-      <c r="E128" s="32" t="s">
+      <c r="F128" s="32" t="s">
         <v>949</v>
-      </c>
-      <c r="F128" s="32" t="s">
-        <v>950</v>
       </c>
       <c r="G128" s="32"/>
       <c r="H128" s="32" t="s">
@@ -17312,7 +17322,7 @@
       <c r="L128" s="31"/>
       <c r="M128" s="32"/>
       <c r="N128" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O128" s="33">
         <v>1</v>
@@ -17396,20 +17406,20 @@
         <v>1</v>
       </c>
       <c r="D129" s="32" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="E129" s="32" t="s">
         <v>35</v>
       </c>
       <c r="F129" s="32" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="G129" s="32"/>
       <c r="H129" s="32" t="s">
         <v>165</v>
       </c>
       <c r="I129" s="31" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="J129" s="31">
         <v>99</v>
@@ -17420,7 +17430,7 @@
       <c r="L129" s="31"/>
       <c r="M129" s="32"/>
       <c r="N129" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O129" s="33">
         <v>1</v>
@@ -17531,7 +17541,7 @@
         <v>8</v>
       </c>
       <c r="M130" s="29" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="N130" s="29"/>
       <c r="O130" s="30"/>
@@ -17620,7 +17630,7 @@
         <v>44</v>
       </c>
       <c r="F131" s="29" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="G131" s="29" t="s">
         <v>130</v>
@@ -17751,10 +17761,10 @@
         <v>11</v>
       </c>
       <c r="M132" s="32" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="N132" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O132" s="33">
         <v>1</v>
@@ -17863,10 +17873,10 @@
         <v>11</v>
       </c>
       <c r="M133" s="32" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="N133" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O133" s="33">
         <v>1</v>
@@ -17978,7 +17988,7 @@
         <v>269</v>
       </c>
       <c r="N134" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O134" s="33">
         <v>1</v>
@@ -18092,7 +18102,7 @@
         <v>499</v>
       </c>
       <c r="N135" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O135" s="33">
         <v>1</v>
@@ -18206,7 +18216,7 @@
         <v>499</v>
       </c>
       <c r="N136" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O136" s="33">
         <v>1</v>
@@ -18296,7 +18306,7 @@
         <v>82</v>
       </c>
       <c r="F137" s="32" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="G137" s="32" t="s">
         <v>93</v>
@@ -18320,7 +18330,7 @@
         <v>269</v>
       </c>
       <c r="N137" s="32" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="O137" s="33">
         <v>1</v>
@@ -18432,7 +18442,7 @@
         <v>269</v>
       </c>
       <c r="N138" s="32" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="O138" s="33">
         <v>1</v>
@@ -18514,13 +18524,13 @@
         <v>1</v>
       </c>
       <c r="D139" s="32" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="E139" s="32" t="s">
         <v>35</v>
       </c>
       <c r="F139" s="32" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="G139" s="32" t="s">
         <v>132</v>
@@ -18529,7 +18539,7 @@
         <v>165</v>
       </c>
       <c r="I139" s="31" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="J139" s="31">
         <v>99</v>
@@ -18540,7 +18550,7 @@
       <c r="L139" s="31"/>
       <c r="M139" s="32"/>
       <c r="N139" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O139" s="33">
         <v>1</v>
@@ -18654,7 +18664,7 @@
         <v>269</v>
       </c>
       <c r="N140" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O140" s="33">
         <v>1</v>
@@ -18744,7 +18754,7 @@
         <v>35</v>
       </c>
       <c r="F141" s="32" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="G141" s="32" t="s">
         <v>521</v>
@@ -18768,7 +18778,7 @@
         <v>269</v>
       </c>
       <c r="N141" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O141" s="33">
         <v>1</v>
@@ -18988,7 +18998,7 @@
         <v>269</v>
       </c>
       <c r="N143" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O143" s="33">
         <v>1</v>
@@ -19073,7 +19083,7 @@
         <v>727</v>
       </c>
       <c r="E144" s="21" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="F144" s="21" t="s">
         <v>728</v>
@@ -19097,7 +19107,7 @@
         <v>35</v>
       </c>
       <c r="M144" s="21" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="N144" s="21"/>
       <c r="O144" s="7"/>
@@ -19205,10 +19215,10 @@
         <v>45</v>
       </c>
       <c r="M145" s="32" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="N145" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O145" s="33">
         <v>1</v>
@@ -19290,11 +19300,11 @@
         <v>2</v>
       </c>
       <c r="D146" s="35" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="E146" s="35"/>
       <c r="F146" s="35" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="G146" s="35" t="s">
         <v>309</v>
@@ -19315,10 +19325,10 @@
         <v>40</v>
       </c>
       <c r="M146" s="35" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="N146" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O146" s="36"/>
       <c r="P146" s="36"/>
@@ -19404,7 +19414,7 @@
         <v>30</v>
       </c>
       <c r="F147" s="32" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="G147" s="32" t="s">
         <v>40</v>
@@ -19428,7 +19438,7 @@
         <v>732</v>
       </c>
       <c r="N147" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O147" s="33">
         <v>1</v>
@@ -19540,7 +19550,7 @@
         <v>40</v>
       </c>
       <c r="N148" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O148" s="33">
         <v>1</v>
@@ -19630,7 +19640,7 @@
         <v>526</v>
       </c>
       <c r="F149" s="32" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="G149" s="32" t="s">
         <v>130</v>
@@ -19652,7 +19662,7 @@
         <v>40</v>
       </c>
       <c r="N149" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O149" s="33">
         <v>1</v>
@@ -19766,7 +19776,7 @@
         <v>337</v>
       </c>
       <c r="N150" s="32" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="O150" s="33">
         <v>1</v>
@@ -19878,7 +19888,7 @@
         <v>337</v>
       </c>
       <c r="N151" s="32" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="O151" s="33">
         <v>1</v>
@@ -19990,7 +20000,7 @@
         <v>749</v>
       </c>
       <c r="N152" s="32" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="O152" s="33">
         <v>1</v>
@@ -20102,7 +20112,7 @@
         <v>603</v>
       </c>
       <c r="N153" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O153" s="36"/>
       <c r="P153" s="36"/>
@@ -20292,10 +20302,10 @@
         <v>2</v>
       </c>
       <c r="D155" s="29" t="s">
+        <v>951</v>
+      </c>
+      <c r="E155" s="29" t="s">
         <v>952</v>
-      </c>
-      <c r="E155" s="29" t="s">
-        <v>953</v>
       </c>
       <c r="F155" s="29" t="s">
         <v>96</v>
@@ -20305,7 +20315,7 @@
         <v>165</v>
       </c>
       <c r="I155" s="28" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="J155" s="28"/>
       <c r="K155" s="28" t="s">
@@ -20424,7 +20434,7 @@
         <v>721</v>
       </c>
       <c r="N156" s="35" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="O156" s="36"/>
       <c r="P156" s="36"/>
@@ -20531,10 +20541,10 @@
         <v>40</v>
       </c>
       <c r="M157" s="32" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="N157" s="32" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="O157" s="33">
         <v>1</v>
@@ -20616,13 +20626,13 @@
         <v>2</v>
       </c>
       <c r="D158" s="35" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="E158" s="35" t="s">
         <v>457</v>
       </c>
       <c r="F158" s="35" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="G158" s="35" t="s">
         <v>676</v>
@@ -20631,7 +20641,7 @@
         <v>165</v>
       </c>
       <c r="I158" s="34" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="J158" s="34">
         <v>99</v>
@@ -20643,10 +20653,10 @@
         <v>20</v>
       </c>
       <c r="M158" s="35" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="N158" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O158" s="36"/>
       <c r="P158" s="36"/>
@@ -20729,10 +20739,10 @@
         <v>725</v>
       </c>
       <c r="E159" s="35" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="F159" s="35" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="G159" s="35" t="s">
         <v>137</v>
@@ -20753,10 +20763,10 @@
         <v>40</v>
       </c>
       <c r="M159" s="35" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="N159" s="35" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="O159" s="36"/>
       <c r="P159" s="36"/>
@@ -20976,7 +20986,7 @@
         <v>40</v>
       </c>
       <c r="N161" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O161" s="33">
         <v>1</v>
@@ -21060,13 +21070,13 @@
         <v>3</v>
       </c>
       <c r="D162" s="32" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="E162" s="32" t="s">
         <v>575</v>
       </c>
       <c r="F162" s="32" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="G162" s="32" t="s">
         <v>38</v>
@@ -21090,7 +21100,7 @@
         <v>270</v>
       </c>
       <c r="N162" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O162" s="33">
         <v>1</v>
@@ -21174,13 +21184,13 @@
         <v>3</v>
       </c>
       <c r="D163" s="32" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="E163" s="32" t="s">
         <v>575</v>
       </c>
       <c r="F163" s="32" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="G163" s="32" t="s">
         <v>160</v>
@@ -21204,7 +21214,7 @@
         <v>270</v>
       </c>
       <c r="N163" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O163" s="33">
         <v>1</v>
@@ -21426,7 +21436,7 @@
         <v>270</v>
       </c>
       <c r="N165" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O165" s="33">
         <v>1</v>
@@ -21510,18 +21520,18 @@
         <v>3</v>
       </c>
       <c r="D166" s="32" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="E166" s="32"/>
       <c r="F166" s="32" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="G166" s="32"/>
       <c r="H166" s="32" t="s">
         <v>165</v>
       </c>
       <c r="I166" s="31" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="J166" s="31"/>
       <c r="K166" s="31" t="s">
@@ -21530,7 +21540,7 @@
       <c r="L166" s="31"/>
       <c r="M166" s="32"/>
       <c r="N166" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O166" s="33">
         <v>1</v>
@@ -21749,10 +21759,10 @@
         <v>35</v>
       </c>
       <c r="M168" s="35" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="N168" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O168" s="36"/>
       <c r="P168" s="36"/>
@@ -21856,13 +21866,13 @@
         <v>320</v>
       </c>
       <c r="L169" s="34" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="M169" s="35" t="s">
         <v>750</v>
       </c>
       <c r="N169" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O169" s="36"/>
       <c r="P169" s="36"/>
@@ -21972,7 +21982,7 @@
         <v>205</v>
       </c>
       <c r="N170" s="35" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="O170" s="36"/>
       <c r="P170" s="36"/>
@@ -22076,13 +22086,13 @@
         <v>318</v>
       </c>
       <c r="L171" s="34" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="M171" s="35" t="s">
         <v>751</v>
       </c>
       <c r="N171" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O171" s="36"/>
       <c r="P171" s="36"/>
@@ -22186,13 +22196,13 @@
         <v>318</v>
       </c>
       <c r="L172" s="34" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="M172" s="35" t="s">
         <v>751</v>
       </c>
       <c r="N172" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O172" s="36"/>
       <c r="P172" s="36"/>
@@ -22278,7 +22288,7 @@
         <v>36</v>
       </c>
       <c r="F173" s="35" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="G173" s="35" t="s">
         <v>107</v>
@@ -22287,7 +22297,7 @@
         <v>165</v>
       </c>
       <c r="I173" s="34" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="J173" s="34">
         <v>99</v>
@@ -22296,13 +22306,13 @@
         <v>318</v>
       </c>
       <c r="L173" s="34" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="M173" s="35" t="s">
         <v>751</v>
       </c>
       <c r="N173" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O173" s="36"/>
       <c r="P173" s="36"/>
@@ -22409,7 +22419,7 @@
         <v>30</v>
       </c>
       <c r="M174" s="40" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="N174" s="21"/>
       <c r="O174" s="7"/>
@@ -22520,7 +22530,7 @@
         <v>702</v>
       </c>
       <c r="N175" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O175" s="36"/>
       <c r="P175" s="36"/>
@@ -22600,22 +22610,22 @@
         <v>4</v>
       </c>
       <c r="D176" s="21" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="E176" s="21" t="s">
         <v>29</v>
       </c>
       <c r="F176" s="21" t="s">
+        <v>829</v>
+      </c>
+      <c r="G176" s="21" t="s">
         <v>830</v>
-      </c>
-      <c r="G176" s="21" t="s">
-        <v>831</v>
       </c>
       <c r="H176" s="21" t="s">
         <v>165</v>
       </c>
       <c r="I176" s="20" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="J176" s="20">
         <v>99</v>
@@ -22843,10 +22853,10 @@
         <v>343</v>
       </c>
       <c r="M178" s="35" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="N178" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O178" s="36"/>
       <c r="P178" s="36"/>
@@ -22916,48 +22926,50 @@
       </c>
     </row>
     <row r="179" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A179" s="34">
-        <v>0</v>
-      </c>
-      <c r="B179" s="34">
+      <c r="A179" s="31">
+        <v>0</v>
+      </c>
+      <c r="B179" s="31">
         <v>2</v>
       </c>
-      <c r="C179" s="34">
+      <c r="C179" s="31">
         <v>4</v>
       </c>
-      <c r="D179" s="35" t="s">
+      <c r="D179" s="32" t="s">
         <v>771</v>
       </c>
-      <c r="E179" s="35" t="s">
+      <c r="E179" s="32" t="s">
         <v>772</v>
       </c>
-      <c r="F179" s="35" t="s">
+      <c r="F179" s="32" t="s">
         <v>773</v>
       </c>
-      <c r="G179" s="35"/>
-      <c r="H179" s="35" t="s">
+      <c r="G179" s="32"/>
+      <c r="H179" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I179" s="34" t="s">
+      <c r="I179" s="31" t="s">
         <v>774</v>
       </c>
-      <c r="J179" s="34">
+      <c r="J179" s="31">
         <v>99</v>
       </c>
-      <c r="K179" s="34" t="s">
+      <c r="K179" s="31" t="s">
         <v>378</v>
       </c>
-      <c r="L179" s="34">
-        <v>30</v>
-      </c>
-      <c r="M179" s="35" t="s">
-        <v>775</v>
-      </c>
-      <c r="N179" s="35" t="s">
-        <v>902</v>
-      </c>
-      <c r="O179" s="36"/>
-      <c r="P179" s="36"/>
+      <c r="L179" s="31">
+        <v>35</v>
+      </c>
+      <c r="M179" s="32" t="s">
+        <v>958</v>
+      </c>
+      <c r="N179" s="32" t="s">
+        <v>906</v>
+      </c>
+      <c r="O179" s="33">
+        <v>1</v>
+      </c>
+      <c r="P179" s="33"/>
       <c r="R179" s="2">
         <f t="shared" si="55"/>
         <v>0</v>
@@ -23004,7 +23016,7 @@
       </c>
       <c r="AD179" s="2">
         <f t="shared" si="66"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE179" s="2">
         <f t="shared" si="51"/>
@@ -23012,7 +23024,7 @@
       </c>
       <c r="AF179" s="2">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG179" s="2">
         <f t="shared" si="53"/>
@@ -23064,7 +23076,7 @@
         <v>706</v>
       </c>
       <c r="N180" s="35" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="O180" s="36"/>
       <c r="P180" s="36"/>
@@ -23174,7 +23186,7 @@
         <v>752</v>
       </c>
       <c r="N181" s="35" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="O181" s="36"/>
       <c r="P181" s="36"/>
@@ -23281,10 +23293,10 @@
         <v>25</v>
       </c>
       <c r="M182" s="35" t="s">
+        <v>934</v>
+      </c>
+      <c r="N182" s="35" t="s">
         <v>935</v>
-      </c>
-      <c r="N182" s="35" t="s">
-        <v>936</v>
       </c>
       <c r="O182" s="36"/>
       <c r="P182" s="36"/>
@@ -23394,7 +23406,7 @@
         <v>500</v>
       </c>
       <c r="N183" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O183" s="36"/>
       <c r="P183" s="36"/>
@@ -23504,7 +23516,7 @@
         <v>606</v>
       </c>
       <c r="N184" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O184" s="36"/>
       <c r="P184" s="36"/>
@@ -23614,7 +23626,7 @@
         <v>756</v>
       </c>
       <c r="N185" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O185" s="33">
         <v>1</v>
@@ -23686,50 +23698,52 @@
       </c>
     </row>
     <row r="186" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A186" s="34">
-        <v>0</v>
-      </c>
-      <c r="B186" s="34">
+      <c r="A186" s="31">
+        <v>0</v>
+      </c>
+      <c r="B186" s="31">
         <v>2</v>
       </c>
-      <c r="C186" s="34">
+      <c r="C186" s="31">
         <v>5</v>
       </c>
-      <c r="D186" s="35" t="s">
+      <c r="D186" s="32" t="s">
         <v>572</v>
       </c>
-      <c r="E186" s="35" t="s">
+      <c r="E186" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="F186" s="35" t="s">
-        <v>833</v>
-      </c>
-      <c r="G186" s="35" t="s">
+      <c r="F186" s="32" t="s">
+        <v>832</v>
+      </c>
+      <c r="G186" s="32" t="s">
         <v>676</v>
       </c>
-      <c r="H186" s="35" t="s">
+      <c r="H186" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I186" s="34" t="s">
+      <c r="I186" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="J186" s="34">
+      <c r="J186" s="31">
         <v>99</v>
       </c>
-      <c r="K186" s="34" t="s">
+      <c r="K186" s="31" t="s">
         <v>320</v>
       </c>
-      <c r="L186" s="34" t="s">
+      <c r="L186" s="31" t="s">
         <v>335</v>
       </c>
-      <c r="M186" s="35" t="s">
+      <c r="M186" s="32" t="s">
         <v>607</v>
       </c>
-      <c r="N186" s="35" t="s">
-        <v>904</v>
-      </c>
-      <c r="O186" s="36"/>
-      <c r="P186" s="36"/>
+      <c r="N186" s="32" t="s">
+        <v>920</v>
+      </c>
+      <c r="O186" s="33">
+        <v>1</v>
+      </c>
+      <c r="P186" s="33"/>
       <c r="R186" s="2">
         <f t="shared" si="55"/>
         <v>0</v>
@@ -23776,7 +23790,7 @@
       </c>
       <c r="AD186" s="2">
         <f t="shared" si="66"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE186" s="2">
         <f t="shared" si="51"/>
@@ -23784,7 +23798,7 @@
       </c>
       <c r="AF186" s="2">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG186" s="2">
         <f t="shared" si="53"/>
@@ -23923,7 +23937,7 @@
         <v>634</v>
       </c>
       <c r="G188" s="35" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="H188" s="35" t="s">
         <v>165</v>
@@ -23941,10 +23955,10 @@
         <v>341</v>
       </c>
       <c r="M188" s="35" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="N188" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O188" s="36"/>
       <c r="P188" s="36"/>
@@ -24024,7 +24038,7 @@
         <v>5</v>
       </c>
       <c r="D189" s="35" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E189" s="35" t="s">
         <v>29</v>
@@ -24054,7 +24068,7 @@
         <v>646</v>
       </c>
       <c r="N189" s="35" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="O189" s="36"/>
       <c r="P189" s="36"/>
@@ -24140,7 +24154,7 @@
         <v>34</v>
       </c>
       <c r="F190" s="35" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="G190" s="35" t="s">
         <v>96</v>
@@ -24164,7 +24178,7 @@
         <v>621</v>
       </c>
       <c r="N190" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O190" s="36"/>
       <c r="P190" s="36"/>
@@ -24259,7 +24273,7 @@
         <v>165</v>
       </c>
       <c r="I191" s="34" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J191" s="34">
         <v>8</v>
@@ -24274,7 +24288,7 @@
         <v>272</v>
       </c>
       <c r="N191" s="35" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="O191" s="36"/>
       <c r="P191" s="36"/>
@@ -24384,7 +24398,7 @@
         <v>704</v>
       </c>
       <c r="N192" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O192" s="36"/>
       <c r="P192" s="36"/>
@@ -24494,7 +24508,7 @@
         <v>753</v>
       </c>
       <c r="N193" s="32" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="O193" s="33">
         <v>1</v>
@@ -24606,7 +24620,7 @@
         <v>705</v>
       </c>
       <c r="N194" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O194" s="36"/>
       <c r="P194" s="36"/>
@@ -24714,7 +24728,7 @@
         <v>272</v>
       </c>
       <c r="N195" s="35" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="O195" s="36"/>
       <c r="P195" s="36"/>
@@ -24824,7 +24838,7 @@
         <v>272</v>
       </c>
       <c r="N196" s="35" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="O196" s="36"/>
       <c r="P196" s="36"/>
@@ -24910,7 +24924,7 @@
         <v>682</v>
       </c>
       <c r="F197" s="35" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="G197" s="35" t="s">
         <v>103</v>
@@ -24919,7 +24933,7 @@
         <v>165</v>
       </c>
       <c r="I197" s="34" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="J197" s="34">
         <v>6</v>
@@ -24934,7 +24948,7 @@
         <v>272</v>
       </c>
       <c r="N197" s="35" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="O197" s="36"/>
       <c r="P197" s="36"/>
@@ -25044,7 +25058,7 @@
         <v>273</v>
       </c>
       <c r="N198" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O198" s="33">
         <v>1</v>
@@ -25128,13 +25142,13 @@
         <v>7</v>
       </c>
       <c r="D199" s="32" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="E199" s="32" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="F199" s="32" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="G199" s="32" t="s">
         <v>132</v>
@@ -25143,7 +25157,7 @@
         <v>165</v>
       </c>
       <c r="I199" s="31" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="J199" s="31">
         <v>99</v>
@@ -25154,7 +25168,7 @@
       <c r="L199" s="31"/>
       <c r="M199" s="32"/>
       <c r="N199" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O199" s="33">
         <v>1</v>
@@ -25228,48 +25242,52 @@
       </c>
     </row>
     <row r="200" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A200" s="20">
-        <v>0</v>
-      </c>
-      <c r="B200" s="20">
+      <c r="A200" s="31">
+        <v>0</v>
+      </c>
+      <c r="B200" s="31">
         <v>2</v>
       </c>
-      <c r="C200" s="20">
+      <c r="C200" s="31">
         <v>7</v>
       </c>
-      <c r="D200" s="21" t="s">
+      <c r="D200" s="32" t="s">
         <v>522</v>
       </c>
-      <c r="E200" s="21" t="s">
+      <c r="E200" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="F200" s="21" t="s">
+      <c r="F200" s="32" t="s">
         <v>523</v>
       </c>
-      <c r="G200" s="21" t="s">
+      <c r="G200" s="32" t="s">
         <v>124</v>
       </c>
-      <c r="H200" s="21" t="s">
+      <c r="H200" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I200" s="20" t="s">
+      <c r="I200" s="31" t="s">
         <v>524</v>
       </c>
-      <c r="J200" s="20">
+      <c r="J200" s="31">
         <v>7</v>
       </c>
-      <c r="K200" s="20" t="s">
+      <c r="K200" s="31" t="s">
         <v>319</v>
       </c>
-      <c r="L200" s="20" t="s">
+      <c r="L200" s="31" t="s">
         <v>318</v>
       </c>
-      <c r="M200" s="21" t="s">
+      <c r="M200" s="32" t="s">
         <v>273</v>
       </c>
-      <c r="N200" s="21"/>
-      <c r="O200" s="7"/>
-      <c r="P200" s="7"/>
+      <c r="N200" s="32" t="s">
+        <v>906</v>
+      </c>
+      <c r="O200" s="33">
+        <v>1</v>
+      </c>
+      <c r="P200" s="33"/>
       <c r="R200" s="2">
         <f t="shared" si="55"/>
         <v>0</v>
@@ -25316,7 +25334,7 @@
       </c>
       <c r="AD200" s="2">
         <f t="shared" si="66"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE200" s="2">
         <f t="shared" si="51"/>
@@ -25324,7 +25342,7 @@
       </c>
       <c r="AF200" s="2">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG200" s="2">
         <f t="shared" si="53"/>
@@ -25376,7 +25394,7 @@
         <v>273</v>
       </c>
       <c r="N201" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O201" s="36"/>
       <c r="P201" s="36"/>
@@ -25486,7 +25504,7 @@
         <v>273</v>
       </c>
       <c r="N202" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O202" s="33">
         <v>1</v>
@@ -25600,7 +25618,7 @@
         <v>273</v>
       </c>
       <c r="N203" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O203" s="33">
         <v>1</v>
@@ -25714,7 +25732,7 @@
         <v>273</v>
       </c>
       <c r="N204" s="32" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="O204" s="33">
         <v>1</v>
@@ -25826,7 +25844,7 @@
         <v>273</v>
       </c>
       <c r="N205" s="32" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="O205" s="33">
         <v>1</v>
@@ -25938,7 +25956,7 @@
         <v>273</v>
       </c>
       <c r="N206" s="32" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="O206" s="33">
         <v>1</v>
@@ -26026,7 +26044,7 @@
         <v>31</v>
       </c>
       <c r="F207" s="35" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="G207" s="35" t="s">
         <v>580</v>
@@ -26050,7 +26068,7 @@
         <v>273</v>
       </c>
       <c r="N207" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O207" s="36"/>
       <c r="P207" s="36"/>
@@ -26160,7 +26178,7 @@
         <v>273</v>
       </c>
       <c r="N208" s="35" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="O208" s="36"/>
       <c r="P208" s="36"/>
@@ -26270,7 +26288,7 @@
         <v>273</v>
       </c>
       <c r="N209" s="35" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="O209" s="36"/>
       <c r="P209" s="36"/>
@@ -26380,7 +26398,7 @@
         <v>273</v>
       </c>
       <c r="N210" s="32" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="O210" s="33">
         <v>1</v>
@@ -26477,7 +26495,7 @@
         <v>165</v>
       </c>
       <c r="I211" s="34" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="J211" s="34">
         <v>3</v>
@@ -26492,7 +26510,7 @@
         <v>273</v>
       </c>
       <c r="N211" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O211" s="36"/>
       <c r="P211" s="36"/>
@@ -26587,7 +26605,7 @@
         <v>165</v>
       </c>
       <c r="I212" s="34" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="J212" s="34">
         <v>6</v>
@@ -26602,7 +26620,7 @@
         <v>273</v>
       </c>
       <c r="N212" s="35" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="O212" s="36"/>
       <c r="P212" s="36"/>
@@ -26712,7 +26730,7 @@
         <v>274</v>
       </c>
       <c r="N213" s="35" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="O213" s="36"/>
       <c r="P213" s="36"/>
@@ -26782,50 +26800,52 @@
       </c>
     </row>
     <row r="214" spans="1:34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A214" s="34">
-        <v>0</v>
-      </c>
-      <c r="B214" s="34">
+      <c r="A214" s="31">
+        <v>0</v>
+      </c>
+      <c r="B214" s="31">
         <v>2</v>
       </c>
-      <c r="C214" s="34">
+      <c r="C214" s="31">
         <v>7</v>
       </c>
-      <c r="D214" s="35" t="s">
+      <c r="D214" s="32" t="s">
         <v>465</v>
       </c>
-      <c r="E214" s="35" t="s">
+      <c r="E214" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="F214" s="35" t="s">
+      <c r="F214" s="32" t="s">
         <v>397</v>
       </c>
-      <c r="G214" s="35" t="s">
+      <c r="G214" s="32" t="s">
         <v>482</v>
       </c>
-      <c r="H214" s="35" t="s">
+      <c r="H214" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I214" s="34" t="s">
+      <c r="I214" s="31" t="s">
         <v>492</v>
       </c>
-      <c r="J214" s="34">
+      <c r="J214" s="31">
         <v>99</v>
       </c>
-      <c r="K214" s="34" t="s">
+      <c r="K214" s="31" t="s">
         <v>378</v>
       </c>
-      <c r="L214" s="34" t="s">
+      <c r="L214" s="31" t="s">
         <v>318</v>
       </c>
-      <c r="M214" s="35" t="s">
+      <c r="M214" s="32" t="s">
         <v>273</v>
       </c>
-      <c r="N214" s="35" t="s">
-        <v>936</v>
-      </c>
-      <c r="O214" s="36"/>
-      <c r="P214" s="36"/>
+      <c r="N214" s="32" t="s">
+        <v>942</v>
+      </c>
+      <c r="O214" s="33">
+        <v>1</v>
+      </c>
+      <c r="P214" s="33"/>
       <c r="R214" s="2">
         <f t="shared" si="71"/>
         <v>0</v>
@@ -26872,7 +26892,7 @@
       </c>
       <c r="AD214" s="2">
         <f t="shared" si="82"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE214" s="2">
         <f t="shared" si="67"/>
@@ -26880,7 +26900,7 @@
       </c>
       <c r="AF214" s="2">
         <f t="shared" si="68"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG214" s="2">
         <f t="shared" si="69"/>
@@ -26932,7 +26952,7 @@
         <v>273</v>
       </c>
       <c r="N215" s="32" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="O215" s="33">
         <v>1</v>
@@ -27014,10 +27034,10 @@
         <v>7</v>
       </c>
       <c r="D216" s="32" t="s">
+        <v>924</v>
+      </c>
+      <c r="E216" s="32" t="s">
         <v>925</v>
-      </c>
-      <c r="E216" s="32" t="s">
-        <v>926</v>
       </c>
       <c r="F216" s="32" t="s">
         <v>146</v>
@@ -27040,7 +27060,7 @@
       <c r="L216" s="31"/>
       <c r="M216" s="32"/>
       <c r="N216" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O216" s="33">
         <v>1</v>
@@ -27124,16 +27144,16 @@
         <v>7</v>
       </c>
       <c r="D217" s="32" t="s">
+        <v>924</v>
+      </c>
+      <c r="E217" s="32" t="s">
         <v>925</v>
       </c>
-      <c r="E217" s="32" t="s">
+      <c r="F217" s="32" t="s">
         <v>926</v>
       </c>
-      <c r="F217" s="32" t="s">
+      <c r="G217" s="32" t="s">
         <v>927</v>
-      </c>
-      <c r="G217" s="32" t="s">
-        <v>928</v>
       </c>
       <c r="H217" s="32" t="s">
         <v>165</v>
@@ -27146,7 +27166,7 @@
       <c r="L217" s="31"/>
       <c r="M217" s="32"/>
       <c r="N217" s="32" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="O217" s="33">
         <v>1</v>
@@ -27260,7 +27280,7 @@
         <v>273</v>
       </c>
       <c r="N218" s="32" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="O218" s="33">
         <v>1</v>
@@ -27372,7 +27392,7 @@
         <v>273</v>
       </c>
       <c r="N219" s="32" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="O219" s="33">
         <v>1</v>
@@ -27484,7 +27504,7 @@
         <v>273</v>
       </c>
       <c r="N220" s="32" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="O220" s="33">
         <v>1</v>
@@ -27596,7 +27616,7 @@
         <v>273</v>
       </c>
       <c r="N221" s="32" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="O221" s="33">
         <v>1</v>
@@ -27708,7 +27728,7 @@
         <v>273</v>
       </c>
       <c r="N222" s="32" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="O222" s="33">
         <v>1</v>
@@ -27820,7 +27840,7 @@
         <v>273</v>
       </c>
       <c r="N223" s="32" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="O223" s="33">
         <v>1</v>
@@ -27932,7 +27952,7 @@
         <v>273</v>
       </c>
       <c r="N224" s="32" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="O224" s="33">
         <v>1</v>
@@ -28044,7 +28064,7 @@
         <v>273</v>
       </c>
       <c r="N225" s="32" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="O225" s="33">
         <v>1</v>
@@ -28156,7 +28176,7 @@
         <v>275</v>
       </c>
       <c r="N226" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O226" s="36"/>
       <c r="P226" s="36"/>
@@ -28266,7 +28286,7 @@
         <v>275</v>
       </c>
       <c r="N227" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O227" s="36"/>
       <c r="P227" s="36"/>
@@ -28376,7 +28396,7 @@
         <v>275</v>
       </c>
       <c r="N228" s="35" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="O228" s="36"/>
       <c r="P228" s="36"/>

</xml_diff>

<commit_message>
chore(mappa): aggiornamento manuale 2026-05-19-0959
</commit_message>
<xml_diff>
--- a/Milano_2027.xlsx
+++ b/Milano_2027.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scarg\Dropbox\PNE Simone\Guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06ECAEF5-64B0-489F-B8CA-20A8F4A14B7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CD6F5A-3FBC-4B54-B127-846079E59B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="665" xr2:uid="{0118EB4B-1337-43BA-A7E3-0EBAC20BAF10}"/>
   </bookViews>
@@ -2865,9 +2865,6 @@
     <t>02/38238682</t>
   </si>
   <si>
-    <t>Via Manzoni, 5</t>
-  </si>
-  <si>
     <t>La Bruma</t>
   </si>
   <si>
@@ -2910,10 +2907,13 @@
     <t>Via Ascanio Sforza, 9</t>
   </si>
   <si>
-    <t>i</t>
-  </si>
-  <si>
     <t>Piazzale Carlo Maciachini, 18</t>
+  </si>
+  <si>
+    <t>Ripa di Porta Ticinese, 43</t>
+  </si>
+  <si>
+    <t>Via Alessandro Manzoni, 5</t>
   </si>
 </sst>
 </file>
@@ -14950,20 +14950,20 @@
         <v>7</v>
       </c>
       <c r="D107" s="21" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="E107" s="21" t="s">
         <v>32</v>
       </c>
       <c r="F107" s="21" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="G107" s="21"/>
       <c r="H107" s="21" t="s">
         <v>165</v>
       </c>
       <c r="I107" s="20" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="J107" s="20"/>
       <c r="K107" s="20" t="s">
@@ -14973,7 +14973,7 @@
         <v>30</v>
       </c>
       <c r="M107" s="21" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="N107" s="21"/>
       <c r="O107" s="7"/>
@@ -15641,7 +15641,7 @@
         <v>6</v>
       </c>
       <c r="M113" s="21" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="N113" s="21"/>
       <c r="O113" s="7"/>
@@ -17300,13 +17300,13 @@
         <v>1</v>
       </c>
       <c r="D128" s="32" t="s">
+        <v>942</v>
+      </c>
+      <c r="E128" s="32" t="s">
         <v>943</v>
       </c>
-      <c r="E128" s="32" t="s">
+      <c r="F128" s="32" t="s">
         <v>944</v>
-      </c>
-      <c r="F128" s="32" t="s">
-        <v>945</v>
       </c>
       <c r="G128" s="32"/>
       <c r="H128" s="32" t="s">
@@ -20088,7 +20088,7 @@
         <v>30</v>
       </c>
       <c r="F153" s="35" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="G153" s="35" t="s">
         <v>580</v>
@@ -20302,10 +20302,10 @@
         <v>2</v>
       </c>
       <c r="D155" s="29" t="s">
+        <v>946</v>
+      </c>
+      <c r="E155" s="29" t="s">
         <v>947</v>
-      </c>
-      <c r="E155" s="29" t="s">
-        <v>948</v>
       </c>
       <c r="F155" s="29" t="s">
         <v>96</v>
@@ -20315,7 +20315,7 @@
         <v>165</v>
       </c>
       <c r="I155" s="28" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="J155" s="28"/>
       <c r="K155" s="28" t="s">
@@ -21076,7 +21076,7 @@
         <v>573</v>
       </c>
       <c r="F162" s="32" t="s">
-        <v>942</v>
+        <v>958</v>
       </c>
       <c r="G162" s="32" t="s">
         <v>38</v>
@@ -22961,7 +22961,7 @@
         <v>35</v>
       </c>
       <c r="M179" s="32" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="N179" s="32" t="s">
         <v>902</v>
@@ -24814,7 +24814,7 @@
         <v>679</v>
       </c>
       <c r="F196" s="35" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="G196" s="35" t="s">
         <v>584</v>
@@ -24924,7 +24924,7 @@
         <v>679</v>
       </c>
       <c r="F197" s="35" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="G197" s="35" t="s">
         <v>103</v>

</xml_diff>